<commit_message>
feat: add end-to-end tests for hierarchy visibility and sibling isolation with updated test data
</commit_message>
<xml_diff>
--- a/client/e2e-test/test-data/contracts.xlsx
+++ b/client/e2e-test/test-data/contracts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="1100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1106" uniqueCount="1106">
   <si>
     <t>Contrato</t>
   </si>
@@ -3110,12 +3110,27 @@
     <t>1100004909</t>
   </si>
   <si>
+    <t>7777</t>
+  </si>
+  <si>
+    <t>Patricia Nível3</t>
+  </si>
+  <si>
     <t>2515</t>
   </si>
   <si>
+    <t>patrician3@example.com</t>
+  </si>
+  <si>
     <t>1100005807</t>
   </si>
   <si>
+    <t>8888</t>
+  </si>
+  <si>
+    <t>Diego Nível4</t>
+  </si>
+  <si>
     <t>1852</t>
   </si>
   <si>
@@ -3123,6 +3138,9 @@
   </si>
   <si>
     <t>Fernando Eduardo Ferreira</t>
+  </si>
+  <si>
+    <t>diegon4@example.com</t>
   </si>
   <si>
     <t>1100005808</t>
@@ -18108,16 +18126,16 @@
         <v>400</v>
       </c>
       <c r="E279" s="0" t="s">
-        <v>40</v>
+        <v>1032</v>
       </c>
       <c r="F279" s="0" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="G279" s="0" t="s">
         <v>55</v>
       </c>
       <c r="H279" s="0" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="I279" s="0" t="s">
         <v>24</v>
@@ -18144,12 +18162,12 @@
         <v>31</v>
       </c>
       <c r="Q279" s="0" t="s">
-        <v>98</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="s">
-        <v>1033</v>
+        <v>1036</v>
       </c>
       <c r="B280" s="0" t="s">
         <v>40</v>
@@ -18161,28 +18179,28 @@
         <v>400</v>
       </c>
       <c r="E280" s="0" t="s">
-        <v>40</v>
+        <v>1037</v>
       </c>
       <c r="F280" s="0" t="s">
-        <v>516</v>
+        <v>1038</v>
       </c>
       <c r="G280" s="0" t="s">
         <v>55</v>
       </c>
       <c r="H280" s="0" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="I280" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J280" s="0" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="K280" s="0" t="s">
         <v>37</v>
       </c>
       <c r="L280" s="0" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="M280" s="0" t="s">
         <v>28</v>
@@ -18197,12 +18215,12 @@
         <v>31</v>
       </c>
       <c r="Q280" s="0" t="s">
-        <v>520</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="0" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="B281" s="0" t="s">
         <v>40</v>
@@ -18223,19 +18241,19 @@
         <v>55</v>
       </c>
       <c r="H281" s="0" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
       <c r="I281" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J281" s="0" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="K281" s="0" t="s">
         <v>37</v>
       </c>
       <c r="L281" s="0" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="M281" s="0" t="s">
         <v>28</v>
@@ -18255,7 +18273,7 @@
     </row>
     <row r="282">
       <c r="A282" s="0" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="B282" s="0" t="s">
         <v>40</v>
@@ -18273,22 +18291,22 @@
         <v>819</v>
       </c>
       <c r="G282" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H282" s="0" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="I282" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J282" s="0" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="K282" s="0" t="s">
         <v>58</v>
       </c>
       <c r="L282" s="0" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="M282" s="0" t="s">
         <v>28</v>
@@ -18308,7 +18326,7 @@
     </row>
     <row r="283">
       <c r="A283" s="0" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
       <c r="B283" s="0" t="s">
         <v>40</v>
@@ -18326,22 +18344,22 @@
         <v>290</v>
       </c>
       <c r="G283" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H283" s="0" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="I283" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J283" s="0" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="K283" s="0" t="s">
         <v>37</v>
       </c>
       <c r="L283" s="0" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="M283" s="0" t="s">
         <v>28</v>
@@ -18361,7 +18379,7 @@
     </row>
     <row r="284">
       <c r="A284" s="0" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
       <c r="B284" s="0" t="s">
         <v>40</v>
@@ -18376,25 +18394,25 @@
         <v>40</v>
       </c>
       <c r="F284" s="0" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="G284" s="0" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
       <c r="H284" s="0" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="I284" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J284" s="0" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="K284" s="0" t="s">
         <v>387</v>
       </c>
       <c r="L284" s="0" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="M284" s="0" t="s">
         <v>28</v>
@@ -18409,12 +18427,12 @@
         <v>31</v>
       </c>
       <c r="Q284" s="0" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="0" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
       <c r="B285" s="0" t="s">
         <v>40</v>
@@ -18432,22 +18450,22 @@
         <v>168</v>
       </c>
       <c r="G285" s="0" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="H285" s="0" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="I285" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J285" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K285" s="0" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
       <c r="L285" s="0" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="M285" s="0" t="s">
         <v>28</v>
@@ -18467,7 +18485,7 @@
     </row>
     <row r="286">
       <c r="A286" s="0" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="B286" s="0" t="s">
         <v>40</v>
@@ -18485,22 +18503,22 @@
         <v>1027</v>
       </c>
       <c r="G286" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H286" s="0" t="s">
-        <v>1061</v>
+        <v>1067</v>
       </c>
       <c r="I286" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J286" s="0" t="s">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="K286" s="0" t="s">
         <v>37</v>
       </c>
       <c r="L286" s="0" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
       <c r="M286" s="0" t="s">
         <v>28</v>
@@ -18520,7 +18538,7 @@
     </row>
     <row r="287">
       <c r="A287" s="0" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="B287" s="0" t="s">
         <v>40</v>
@@ -18541,19 +18559,19 @@
         <v>839</v>
       </c>
       <c r="H287" s="0" t="s">
-        <v>1065</v>
+        <v>1071</v>
       </c>
       <c r="I287" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J287" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K287" s="0" t="s">
         <v>152</v>
       </c>
       <c r="L287" s="0" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="M287" s="0" t="s">
         <v>28</v>
@@ -18573,7 +18591,7 @@
     </row>
     <row r="288">
       <c r="A288" s="0" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="B288" s="0" t="s">
         <v>40</v>
@@ -18585,7 +18603,7 @@
         <v>400</v>
       </c>
       <c r="E288" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="F288" s="0" t="s">
         <v>819</v>
@@ -18600,13 +18618,13 @@
         <v>24</v>
       </c>
       <c r="J288" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K288" s="0" t="s">
         <v>710</v>
       </c>
       <c r="L288" s="0" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="M288" s="0" t="s">
         <v>28</v>
@@ -18626,7 +18644,7 @@
     </row>
     <row r="289">
       <c r="A289" s="0" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="B289" s="0" t="s">
         <v>40</v>
@@ -18638,7 +18656,7 @@
         <v>400</v>
       </c>
       <c r="E289" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="F289" s="0" t="s">
         <v>819</v>
@@ -18653,13 +18671,13 @@
         <v>24</v>
       </c>
       <c r="J289" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K289" s="0" t="s">
         <v>710</v>
       </c>
       <c r="L289" s="0" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="M289" s="0" t="s">
         <v>28</v>
@@ -18679,7 +18697,7 @@
     </row>
     <row r="290">
       <c r="A290" s="0" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="B290" s="0" t="s">
         <v>40</v>
@@ -18691,7 +18709,7 @@
         <v>400</v>
       </c>
       <c r="E290" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="F290" s="0" t="s">
         <v>819</v>
@@ -18706,13 +18724,13 @@
         <v>24</v>
       </c>
       <c r="J290" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K290" s="0" t="s">
         <v>710</v>
       </c>
       <c r="L290" s="0" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="M290" s="0" t="s">
         <v>28</v>
@@ -18732,19 +18750,19 @@
     </row>
     <row r="291">
       <c r="A291" s="0" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
       <c r="B291" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C291" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D291" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E291" s="0" t="s">
         <v>1074</v>
-      </c>
-      <c r="D291" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E291" s="0" t="s">
-        <v>1068</v>
       </c>
       <c r="F291" s="0" t="s">
         <v>819</v>
@@ -18753,19 +18771,19 @@
         <v>999</v>
       </c>
       <c r="H291" s="0" t="s">
-        <v>1076</v>
+        <v>1082</v>
       </c>
       <c r="I291" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J291" s="0" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="K291" s="0" t="s">
         <v>710</v>
       </c>
       <c r="L291" s="0" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="M291" s="0" t="s">
         <v>28</v>
@@ -18785,40 +18803,40 @@
     </row>
     <row r="292">
       <c r="A292" s="0" t="s">
-        <v>1077</v>
+        <v>1083</v>
       </c>
       <c r="B292" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C292" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D292" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E292" s="0" t="s">
         <v>1074</v>
-      </c>
-      <c r="D292" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E292" s="0" t="s">
-        <v>1068</v>
       </c>
       <c r="F292" s="0" t="s">
         <v>366</v>
       </c>
       <c r="G292" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H292" s="0" t="s">
-        <v>1078</v>
+        <v>1084</v>
       </c>
       <c r="I292" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J292" s="0" t="s">
-        <v>1079</v>
+        <v>1085</v>
       </c>
       <c r="K292" s="0" t="s">
         <v>58</v>
       </c>
       <c r="L292" s="0" t="s">
-        <v>1080</v>
+        <v>1086</v>
       </c>
       <c r="M292" s="0" t="s">
         <v>28</v>
@@ -18838,40 +18856,40 @@
     </row>
     <row r="293">
       <c r="A293" s="0" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B293" s="0" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C293" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D293" s="0" t="s">
         <v>1081</v>
       </c>
-      <c r="B293" s="0" t="s">
-        <v>1068</v>
-      </c>
-      <c r="C293" s="0" t="s">
+      <c r="E293" s="0" t="s">
         <v>1074</v>
-      </c>
-      <c r="D293" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E293" s="0" t="s">
-        <v>1068</v>
       </c>
       <c r="F293" s="0" t="s">
         <v>968</v>
       </c>
       <c r="G293" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H293" s="0" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
       <c r="I293" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J293" s="0" t="s">
-        <v>1079</v>
+        <v>1085</v>
       </c>
       <c r="K293" s="0" t="s">
         <v>300</v>
       </c>
       <c r="L293" s="0" t="s">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="M293" s="0" t="s">
         <v>28</v>
@@ -18891,7 +18909,7 @@
     </row>
     <row r="294">
       <c r="A294" s="0" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="B294" s="0" t="s">
         <v>40</v>
@@ -18903,7 +18921,7 @@
         <v>400</v>
       </c>
       <c r="E294" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="F294" s="0" t="s">
         <v>168</v>
@@ -18912,19 +18930,19 @@
         <v>999</v>
       </c>
       <c r="H294" s="0" t="s">
-        <v>1085</v>
+        <v>1091</v>
       </c>
       <c r="I294" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J294" s="0" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="K294" s="0" t="s">
         <v>360</v>
       </c>
       <c r="L294" s="0" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
       <c r="M294" s="0" t="s">
         <v>28</v>
@@ -18944,40 +18962,40 @@
     </row>
     <row r="295">
       <c r="A295" s="0" t="s">
-        <v>1088</v>
+        <v>1094</v>
       </c>
       <c r="B295" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C295" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D295" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E295" s="0" t="s">
         <v>1074</v>
-      </c>
-      <c r="D295" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E295" s="0" t="s">
-        <v>1068</v>
       </c>
       <c r="F295" s="0" t="s">
         <v>930</v>
       </c>
       <c r="G295" s="0" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="H295" s="0" t="s">
-        <v>1089</v>
+        <v>1095</v>
       </c>
       <c r="I295" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J295" s="0" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="K295" s="0" t="s">
         <v>58</v>
       </c>
       <c r="L295" s="0" t="s">
-        <v>1090</v>
+        <v>1096</v>
       </c>
       <c r="M295" s="0" t="s">
         <v>28</v>
@@ -18997,40 +19015,40 @@
     </row>
     <row r="296">
       <c r="A296" s="0" t="s">
-        <v>1091</v>
+        <v>1097</v>
       </c>
       <c r="B296" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C296" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D296" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E296" s="0" t="s">
         <v>1074</v>
       </c>
-      <c r="D296" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E296" s="0" t="s">
-        <v>1068</v>
-      </c>
       <c r="F296" s="0" t="s">
+        <v>1098</v>
+      </c>
+      <c r="G296" s="0" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H296" s="0" t="s">
+        <v>1099</v>
+      </c>
+      <c r="I296" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="J296" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="G296" s="0" t="s">
-        <v>1040</v>
-      </c>
-      <c r="H296" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="I296" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="J296" s="0" t="s">
-        <v>1086</v>
       </c>
       <c r="K296" s="0" t="s">
         <v>58</v>
       </c>
       <c r="L296" s="0" t="s">
-        <v>1094</v>
+        <v>1100</v>
       </c>
       <c r="M296" s="0" t="s">
         <v>28</v>
@@ -19045,24 +19063,24 @@
         <v>31</v>
       </c>
       <c r="Q296" s="0" t="s">
-        <v>1095</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="0" t="s">
-        <v>1096</v>
+        <v>1102</v>
       </c>
       <c r="B297" s="0" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C297" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D297" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E297" s="0" t="s">
         <v>1074</v>
-      </c>
-      <c r="D297" s="0" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E297" s="0" t="s">
-        <v>1068</v>
       </c>
       <c r="F297" s="0" t="s">
         <v>394</v>
@@ -19071,19 +19089,19 @@
         <v>839</v>
       </c>
       <c r="H297" s="0" t="s">
-        <v>1097</v>
+        <v>1103</v>
       </c>
       <c r="I297" s="0" t="s">
         <v>24</v>
       </c>
       <c r="J297" s="0" t="s">
-        <v>1098</v>
+        <v>1104</v>
       </c>
       <c r="K297" s="0" t="s">
         <v>152</v>
       </c>
       <c r="L297" s="0" t="s">
-        <v>1099</v>
+        <v>1105</v>
       </c>
       <c r="M297" s="0" t="s">
         <v>28</v>

</xml_diff>